<commit_message>
descarga las 181 series sin problemas
</commit_message>
<xml_diff>
--- a/Codigos.xlsx
+++ b/Codigos.xlsx
@@ -9,7 +9,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -42,7 +42,9 @@
       <family val="2"/>
       <sz val="11"/>
     </font>
-    <font/>
+    <font>
+      <color rgb="00000000"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -64,12 +66,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -413,15 +421,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="32.44140625" customWidth="1" style="2" min="1" max="1"/>
     <col width="32.88671875" customWidth="1" style="2" min="2" max="2"/>
     <col width="24.21875" customWidth="1" style="2" min="3" max="3"/>
     <col width="23.44140625" customWidth="1" style="2" min="4" max="4"/>
-    <col width="8.88671875" customWidth="1" style="2" min="5" max="6"/>
-    <col width="8.88671875" customWidth="1" style="2" min="7" max="16384"/>
+    <col width="8.88671875" customWidth="1" style="2" min="5" max="11"/>
+    <col width="8.88671875" customWidth="1" style="2" min="12" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="1">
@@ -447,1586 +455,3987 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>42.1_EPAT_0_A_27</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Tasa de actividad</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>EPH A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>42.1_EPET_0_A_24</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Tasa de empleo</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>EPH A</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>42.1_EPDT_0_A_30</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>Tasa de desocupación</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>EPH A</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>42.1_EPST_0_A_30</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Tasa de subocupación</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>EPH A</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>49.1_TAEP_0_0_37</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Población Total</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="5" t="inlineStr">
         <is>
           <t>49.1_TAEP_0_0_25</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>PEA</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="5" t="inlineStr">
         <is>
           <t>49.1_TAEO_0_0_30</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>Ocupados</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>49.1_TAED_0_0_33</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Desocupados</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>49.1_TOTAL_AGLODOS_0_S_33_15</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>Subocupados</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>49.1_TOTAL_AGLOTES_0_S_45_28</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Subocupados Demandantes</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>49.1_TOTAL_AGLOTES_0_S_48_98</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>Subocupados No Demandantes</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones S</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
         <is>
           <t>49.2_TAEP_0_0_37</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Población Total</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="5" t="inlineStr">
         <is>
           <t>49.2_TAEP_0_0_25</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>PEA</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>49.2_TAEO_0_0_30</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Ocupados</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>49.2_TAED_0_0_33</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>Desocupados</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>49.2_TOTAL_AGLODOS_0_T_33_90</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>Subocupados</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>49.2_TOTAL_AGLOTES_0_T_45_1</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>Subocupados Demandantes</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>49.2_TOTAL_AGLOTES_0_T_48_13</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>Subocupados No Demandantes</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>EPH-Poblaciones T</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>50.1_IT_0_0_12</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>Evolución del empleo total</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>EIL-Sector A</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>50.1_II_0_0_16</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>Evolución del empleo Industria</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>EIL-Sector A</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>50.1_IC_0_0_19</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>Evolución del empleo Construcción</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>EIL-Sector A</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>50.1_ICS_0_0_25</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Evolución del empleo Comercio y Servicios</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>EIL-Sector A</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
         <is>
           <t>56.1_NGMD_2012_T_22</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Índices de Salarios, nivel general</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>IS T</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
+      <c r="B25" s="5" t="inlineStr">
         <is>
           <t>158.1_REPTE_0_0_5</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Remuneración imponible promedio de los trabajadores estables</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>RIPTE M</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>57.1_SMVMM_0_M_34</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Salario Mínimo Vital y Movil</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>SMVM M</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>58.1_MP_0_M_24</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Haber mínimo jubilatorio $ corrientes</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>HaberMin M</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>60.1_IH_0_0_18</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C28" s="5" t="inlineStr">
         <is>
           <t>Evolución de Hogares, Indigentes</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="5" t="inlineStr">
         <is>
           <t>EPH Puntual - Pel M</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>60.1_PH_0_0_14</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Evolución de Hogares, Pobres</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>EPH Puntual - Pel M</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>60.1_IP_0_0_20</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>Evolución de Personas, Indigentes</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>EPH Puntual - Pel M</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>Empleo e Ingresos: Apendice3A</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>60.1_PP_0_0_15</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Evolución de Personas, Pobres</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>EPH Puntual - Pel M</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>145.1_IPC_NG_NACNAL_DICI_T_15</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>IPC Nivel General (m)</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>IPC Mensual M</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>147.1_IPC_BIENESNAL_DICI_T_19</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>IPC Bienes (m)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>IPC Mensual M</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>147.1_IPC_SERVICNAL_DICI_T_22</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>IPC Servicios (m)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>IPC Mensual M</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>148.1_IPC_NIVEL_NAL_DICI_T_26</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>IPC Categorías-Nivel general (m)</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>IPC Mensual M</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>114.1_CPA_0_0_25</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Cotizacion Peso argentino (d)</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>TCN D</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>116.1_TCRMA_0_A_36</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Índice de Tipo de Cambio Real Multilateral. Diciembre 2015=100 (d)</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>ITCRM D</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>117.1_ENGV_0_A_33</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Índice de valor de las exportaciones de bienes. 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>EXPO IMPO P Y Q T</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>117.1_ENGC_0_A_36</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Índice de cantidad de las exportaciones de bienes. 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>EXPO IMPO P Y Q T</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>118.1_INGV_0_A_33</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Índice de valor de las importaciones de bienes 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>EXPO IMPO P Y Q T</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>118.1_INGC_0_A_36</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Índice de cantidad de las importaciones de bienes 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>EXPO IMPO P Y Q T</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>119.1_IPE_0_A_26</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Índice de precios de exportación. 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>EXPO IMPO P Y Q T</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>119.1_IPI_0_A_26</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>Índice de precio de importación de bienes 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>EXPO IMPO P Y Q T</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>119.1_TI_0_A_20</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Índice de Términos del Intercambio. 2004=100 (t)</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>TDI T</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>110.1_IPC_1993_A_17</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>Índice de precios Implícitos en el PIB corriente. 1993=100 (t)</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>IPI T</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>111.1_IPB_1993_A_14</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Índice de precios implícitos en el PIB de sectores productores de bienes (t)</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>IPI T</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>111.1_IPS_1993_A_17</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Índice de precios implícitos en el PIB de sectores productores de servicios (t)</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>IPI T</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>115.1_TCRM_0_A_29</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Índice de Tipo de Cambio Real Multilateral (m)</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>ITCRM M</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>430.1_REM_IPC_NAL_T_M_0_0_25_28</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr">
+        <is>
+          <t>Relevamiento de Expectativas de Mercado (REM). Var % mensual en t. (m)</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>EXP INF M</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>Precios: Apendice4</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>431.1_EXPECTATIVDIO_M_0_0_30_56</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Expectativas de Inflación (Di Tella). Promedio (m)</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>EXP INF M</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas: Apendice-Financiero</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>169.1_MALVAL_0_0_6</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr">
+        <is>
+          <t>Índice Merval (d)</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>1. Renta Variable D</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas: Apendice-Financiero</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
+        <is>
+          <t>168.1_T_CAMBI500_D_0_0_17</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de cambio mayorista de referencia (d)</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>2. Mercado Cambiario D</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas: Apendice-Financiero</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>168.1_T_CAMBIOR_D_0_0_26</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio BNA (Vendedor) (d)</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>2. Mercado Cambiario D</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>379.1_RESULTADO_006__23_58</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Resultado Financiero (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>379.2_RESULTADO_014__23_28</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr">
+        <is>
+          <t>Resultado Financiero (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>379.3_RESULTADO_017__18_83</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Resultado Financiero(desde 2015)</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>398.1_RESULTADO_ERO_DEVE_A_20_94</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Resultado financiero devengado (1993-2018)</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>SPA_DEV_93 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B58" s="5" t="inlineStr">
+        <is>
+          <t>379.1_ING_ANTES_006__31_92</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos antes de figurativos (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D58" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>379.2_ING_ANTES_014__31_66</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos antes de figurativos (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>379.3_ING_ANTES_017__26_5</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos antes de figurativos (2015-2025)</t>
+        </is>
+      </c>
+      <c r="D60" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>379.1_GTOS_ANTES006__32_18</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Gastos antes de figurativos (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr">
+        <is>
+          <t>379.2_GTOS_ANTES014__32_67</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Gastos antes de figurativos (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>379.3_GTOS_ANTES017__27_95</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Gastos antes de figurativos (2015-2025)</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>379.1_SUPERAVIT_006__28_89</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Superavit primario (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>379.2_SUPERAVIT_014__28_63</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Superavit primario (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B66" s="5" t="inlineStr">
+        <is>
+          <t>379.3_SUPERAVIT_017__23_25</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Superavit primario (desde 2015)</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>SPN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>142.1_GANAN_2001_A_9</t>
+        </is>
+      </c>
+      <c r="C67" s="5" t="inlineStr">
+        <is>
+          <t>Recaudación ganancias</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>RECA - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>142.1_IVA_2001_A_3</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>IVA</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>RECA - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>142.1_CREDI_2001_A_24</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>Créditos y débitos en C/C</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>RECA - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>172.1_SRIDAD_IAL_0_0_16</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Sistema de seguridad social</t>
+        </is>
+      </c>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>RECA_SUB A</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>142.1_DEREC_2001_A_20</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Derechos de exportación</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>RECA A</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>142.1_DEREC_2001_A_26</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Derechos de importación</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>RECA - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>172.1_TL_RECAION_0_0_17</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Total recursos tributarios</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>RECA_SUB - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr">
+        <is>
+          <t>452.2_GANANCIASIAS_0_T_9_12</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Ganancias</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>IMIG - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>429.1_RECAUDACIO969_A_0_0_38_99</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Recaudacion historia impuestos (1932-1969)</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>RECA_HISTORICA - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr">
+        <is>
+          <t>186.1_TOTAL_POLISOS_0_0_23</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Total gasto por politicas de ingresos (2004-2025)</t>
+        </is>
+      </c>
+      <c r="D76" s="5" t="inlineStr">
+        <is>
+          <t>Gasto Pol. Ingreso A</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>187.1_TOTAL_JUBIINO_0_0_58</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>Jubilaciones + Pensiones</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>JUB; PNC; SEG DES. A</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr">
+        <is>
+          <t>463.1_AUH_ASIGNA019_0_M_66_38</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>AUH (Agosto 19 - Hoy)</t>
+        </is>
+      </c>
+      <c r="D78" s="5" t="inlineStr">
+        <is>
+          <t>AUH - AUE M</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>372.1_ING_ANTES_006__31_56</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos antes de figurativos (1993-2005)</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>372.2_ING_ANTES_014__31_61</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos antes de figurativos (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>372.3_ING_ANTES_017__26_97</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Ingresos antes de figurativos (2015-2025)</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>372.1_GTOS_ANTES006__32_78</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Gastos antes de figurativos (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>372.2_GTOS_ANTES014__32_40</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>Gastos antes de figurativos (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>372.3_GTOS_ANTES017__27_1</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr">
+        <is>
+          <t>Gastos antes de figurativos (2015-2025)</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>372.1_SUPERAVIT_006__28_10</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>Superavit primario (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
+        <is>
+          <t>372.2_SUPERAVIT_014__28_86</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Superavit primario (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D86" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>372.3_SUPERAVIT_017__23_94</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>Superavit primario (desde 2015)</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B88" s="5" t="inlineStr">
+        <is>
+          <t>372.1_RESULTADO_006__23_78</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr">
+        <is>
+          <t>Resultado Financiero (1993-2006)</t>
+        </is>
+      </c>
+      <c r="D88" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>372.2_RESULTADO_014__23_16</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>Resultado Financiero (2007-2014)</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
+        <is>
+          <t>Finanzas Públicas: Apendice6</t>
+        </is>
+      </c>
+      <c r="B90" s="5" t="inlineStr">
+        <is>
+          <t>372.3_RESULTADO_017__18_43</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Resultado Financiero(desde 2015)</t>
+        </is>
+      </c>
+      <c r="D90" s="5" t="inlineStr">
+        <is>
+          <t>APN - A</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B91" s="5" t="inlineStr">
         <is>
           <t>4.1_OGP_2004_A_17</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C91" s="5" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B92" s="5" t="inlineStr">
         <is>
           <t>4.1_OGI_2004_A_25</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C92" s="5" t="inlineStr">
         <is>
           <t>Importaciones</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D92" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
+      <c r="B93" s="5" t="inlineStr">
         <is>
           <t>4.1_MGCP_2004_A_25</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
         <is>
           <t>Consumo Privado</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B94" s="5" t="inlineStr">
         <is>
           <t>4.1_DGCP_2004_A_30</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C94" s="5" t="inlineStr">
         <is>
           <t>Consumo Público</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D94" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
+      <c r="B95" s="5" t="inlineStr">
         <is>
           <t>4.1_DGIT_2004_A_25</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C95" s="5" t="inlineStr">
         <is>
           <t>Inversión bruta interna fija</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D95" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B96" s="5" t="inlineStr">
         <is>
           <t>4.1_DGE_2004_A_26</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C96" s="5" t="inlineStr">
         <is>
           <t>Exportaciones</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D96" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B97" s="5" t="inlineStr">
         <is>
           <t>4.1_VE_2004_A_21</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C97" s="5" t="inlineStr">
         <is>
           <t>Variación de Existencias</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B98" s="5" t="inlineStr">
         <is>
           <t>4.1_DE_2004_A_24</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C98" s="5" t="inlineStr">
         <is>
           <t>Discrepancia Estadística</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D98" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
+      <c r="B99" s="5" t="inlineStr">
         <is>
           <t>4.2_OGP_2004_T_17</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C99" s="5" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D99" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B100" s="5" t="inlineStr">
         <is>
           <t>4.2_OGI_2004_T_25</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C100" s="5" t="inlineStr">
         <is>
           <t>Importaciones</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D100" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B101" s="5" t="inlineStr">
         <is>
           <t>4.2_MGCP_2004_T_25</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C101" s="5" t="inlineStr">
         <is>
           <t>Consumo Privado</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D101" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B102" s="5" t="inlineStr">
         <is>
           <t>4.2_DGCP_2004_T_30</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C102" s="5" t="inlineStr">
         <is>
           <t>Consumo Público</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D102" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B103" s="5" t="inlineStr">
         <is>
           <t>4.2_DGIT_2004_T_25</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C103" s="5" t="inlineStr">
         <is>
           <t>Inversión bruta interna fija</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D103" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B104" s="5" t="inlineStr">
         <is>
           <t>4.2_DGE_2004_T_26</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C104" s="5" t="inlineStr">
         <is>
           <t>Exportaciones</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D104" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
+      <c r="B105" s="5" t="inlineStr">
         <is>
           <t>4.2_VE_2004_T_21</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C105" s="5" t="inlineStr">
         <is>
           <t>Variación de Existencias</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D105" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B106" s="5" t="inlineStr">
         <is>
           <t>4.2_DE_2004_T_24</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
         <is>
           <t>Discrepancia Estadística</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D106" s="5" t="inlineStr">
         <is>
           <t>1.1.1 OyD real BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
         <is>
           <t>3.1_OGP_D_2004_A_17</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C107" s="5" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D107" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B108" s="5" t="inlineStr">
         <is>
           <t>3.1_OGI_D_2004_A_25</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C108" s="5" t="inlineStr">
         <is>
           <t>Importaciones</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D108" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B109" s="5" t="inlineStr">
         <is>
           <t>3.1_DGE_D_2004_A_26</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C109" s="5" t="inlineStr">
         <is>
           <t>Exportaciones</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D109" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="4" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B51" s="4" t="inlineStr">
+      <c r="B110" s="5" t="inlineStr">
         <is>
           <t>3.1_DGI_D_2004_A_19</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
+      <c r="C110" s="5" t="inlineStr">
         <is>
           <t>Inversión bruta interna fija</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D110" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B111" s="5" t="inlineStr">
         <is>
           <t>3.1_DGCP_D_2004_A_27</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C111" s="5" t="inlineStr">
         <is>
           <t>Consumo Público</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D111" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B53" s="4" t="inlineStr">
+      <c r="B112" s="5" t="inlineStr">
         <is>
           <t>3.1_DGCP_D_2004_A_30</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
+      <c r="C112" s="5" t="inlineStr">
         <is>
           <t>Consumo Privado</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D112" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B113" s="5" t="inlineStr">
         <is>
           <t>3.2_OGP_D_2004_T_17</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C113" s="5" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D113" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B114" s="5" t="inlineStr">
         <is>
           <t>3.2_OGI_D_2004_T_25</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C114" s="5" t="inlineStr">
         <is>
           <t>Importaciones</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D114" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr">
         <is>
           <t>3.2_DGE_D_2004_T_26</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C115" s="5" t="inlineStr">
         <is>
           <t>Exportaciones</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D115" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="4" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B57" s="4" t="inlineStr">
+      <c r="B116" s="5" t="inlineStr">
         <is>
           <t>3.2_DGI_D_2004_T_19</t>
         </is>
       </c>
-      <c r="C57" s="4" t="inlineStr">
+      <c r="C116" s="5" t="inlineStr">
         <is>
           <t>Inversión bruta interna fija</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D116" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B117" s="5" t="inlineStr">
         <is>
           <t>3.2_DGCP_D_2004_T_27</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C117" s="5" t="inlineStr">
         <is>
           <t>Consumo Público</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D117" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B118" s="5" t="inlineStr">
         <is>
           <t>3.2_DGCP_D_2004_T_30</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C118" s="5" t="inlineStr">
         <is>
           <t>Consumo Privado</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D118" s="5" t="inlineStr">
         <is>
           <t>1.2.1 OyD real s.e. BASE 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B119" s="5" t="inlineStr">
         <is>
           <t>143.3_NO_PR_2004_A_21</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C119" s="5" t="inlineStr">
         <is>
           <t>Original</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D119" s="5" t="inlineStr">
         <is>
           <t>1.4.1 Emae BASE 2004 M</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
+      <c r="B120" s="5" t="inlineStr">
         <is>
           <t>143.3_NO_PR_2004_A_31</t>
         </is>
       </c>
-      <c r="C61" s="4" t="inlineStr">
+      <c r="C120" s="5" t="inlineStr">
         <is>
           <t>Desestacionalizado</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D120" s="5" t="inlineStr">
         <is>
           <t>1.4.1 Emae BASE 2004 M</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B121" s="5" t="inlineStr">
         <is>
           <t>4.3_OGP_2004_A_17</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C121" s="5" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D121" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="4" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B63" s="4" t="inlineStr">
+      <c r="B122" s="5" t="inlineStr">
         <is>
           <t>4.3_OGI_2004_A_25</t>
         </is>
       </c>
-      <c r="C63" s="4" t="inlineStr">
+      <c r="C122" s="5" t="inlineStr">
         <is>
           <t>Importaciones</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D122" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B123" s="5" t="inlineStr">
         <is>
           <t>4.3_DGCP_2004_A_27</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C123" s="5" t="inlineStr">
         <is>
           <t>Consumo Privado</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D123" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="4" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B65" s="4" t="inlineStr">
+      <c r="B124" s="5" t="inlineStr">
         <is>
           <t>4.3_DGCP_2004_A_30</t>
         </is>
       </c>
-      <c r="C65" s="4" t="inlineStr">
+      <c r="C124" s="5" t="inlineStr">
         <is>
           <t>Consumo Público</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="D124" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
+      <c r="B125" s="5" t="inlineStr">
         <is>
           <t>4.3_DGI_2004_A_19</t>
         </is>
       </c>
-      <c r="C66" s="4" t="inlineStr">
+      <c r="C125" s="5" t="inlineStr">
         <is>
           <t>Inversión bruta interna fija</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D125" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="4" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B67" s="4" t="inlineStr">
+      <c r="B126" s="5" t="inlineStr">
         <is>
           <t>4.3_DGE_2004_A_26</t>
         </is>
       </c>
-      <c r="C67" s="4" t="inlineStr">
+      <c r="C126" s="5" t="inlineStr">
         <is>
           <t>Exportaciones</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D126" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 A</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+    <row r="127">
+      <c r="A127" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
+      <c r="B127" s="5" t="inlineStr">
         <is>
           <t>4.4_OGP_2004_T_17</t>
         </is>
       </c>
-      <c r="C68" s="4" t="inlineStr">
+      <c r="C127" s="5" t="inlineStr">
         <is>
           <t>PIB</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D127" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="4" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B69" s="4" t="inlineStr">
+      <c r="B128" s="5" t="inlineStr">
         <is>
           <t>4.4_OGI_2004_T_25</t>
         </is>
       </c>
-      <c r="C69" s="4" t="inlineStr">
+      <c r="C128" s="5" t="inlineStr">
         <is>
           <t>Importaciones</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D128" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B70" s="4" t="inlineStr">
+      <c r="B129" s="5" t="inlineStr">
         <is>
           <t>4.4_DGCP_2004_T_27</t>
         </is>
       </c>
-      <c r="C70" s="4" t="inlineStr">
+      <c r="C129" s="5" t="inlineStr">
         <is>
           <t>Consumo Privado</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
+      <c r="D129" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="4" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B71" s="4" t="inlineStr">
+      <c r="B130" s="5" t="inlineStr">
         <is>
           <t>4.4_DGCP_2004_T_30</t>
         </is>
       </c>
-      <c r="C71" s="4" t="inlineStr">
+      <c r="C130" s="5" t="inlineStr">
         <is>
           <t>Consumo Público</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
+      <c r="D130" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="4" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B72" s="4" t="inlineStr">
+      <c r="B131" s="5" t="inlineStr">
         <is>
           <t>4.4_DGI_2004_T_19</t>
         </is>
       </c>
-      <c r="C72" s="4" t="inlineStr">
+      <c r="C131" s="5" t="inlineStr">
         <is>
           <t>Inversión bruta interna fija</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="D131" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 T</t>
         </is>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="4" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="5" t="inlineStr">
         <is>
           <t>Actividad: Actividad_IED</t>
         </is>
       </c>
-      <c r="B73" s="4" t="inlineStr">
+      <c r="B132" s="5" t="inlineStr">
         <is>
           <t>4.4_DGE_2004_T_26</t>
         </is>
       </c>
-      <c r="C73" s="4" t="inlineStr">
+      <c r="C132" s="5" t="inlineStr">
         <is>
           <t>Exportaciones</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D132" s="5" t="inlineStr">
         <is>
           <t>1.5.1 OyD corr. 2004 T</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>74.1_IET_0_A_16</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>ICA A</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B134" s="5" t="inlineStr">
+        <is>
+          <t>74.2_IET_0_T_16</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D134" s="5" t="inlineStr">
+        <is>
+          <t>ICA T</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>74.3_IET_0_M_16</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>ICA M</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B136" s="5" t="inlineStr">
+        <is>
+          <t>74.1_IIT_0_A_25</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D136" s="5" t="inlineStr">
+        <is>
+          <t>ICA A</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>74.2_IIT_0_T_25</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>ICA T</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B138" s="5" t="inlineStr">
+        <is>
+          <t>74.3_IIT_0_M_25</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D138" s="5" t="inlineStr">
+        <is>
+          <t>ICA M</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>160.1_CTA_CORFOB_0_A_59</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B140" s="5" t="inlineStr">
+        <is>
+          <t>160.1_CTA_CORIOS_0_A_52</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de servicios en USD</t>
+        </is>
+      </c>
+      <c r="D140" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>160.1_CTA_CORRFOB_0_A_59</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>160.1_CTA_CORIOS_0_A_51</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de servicios en USD</t>
+        </is>
+      </c>
+      <c r="D142" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>160.1_TL_CUENNTE_0_A_22</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>Cuenta Corriente en USD</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B144" s="5" t="inlineStr">
+        <is>
+          <t>160.1_TL_CUENERA_0_A_23</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>Cuenta Financiera en USD</t>
+        </is>
+      </c>
+      <c r="D144" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>160.1_AVOS_RERVA_0_A_15</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>Activos de Reserva en USD</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS A</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B146" s="5" t="inlineStr">
+        <is>
+          <t>160.2_CTA_CORFOB_0_T_59</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D146" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>160.2_CTA_CORIOS_0_T_52</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>Exportaciones de servicios en USD</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B148" s="5" t="inlineStr">
+        <is>
+          <t>160.2_CTA_CORRFOB_0_T_59</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de bienes en USD</t>
+        </is>
+      </c>
+      <c r="D148" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>160.2_CTA_CORIOS_0_T_51</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>Importaciones de servicios en USD</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B150" s="5" t="inlineStr">
+        <is>
+          <t>160.2_TL_CUENNTE_0_T_22</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>Cuenta Corriente en USD</t>
+        </is>
+      </c>
+      <c r="D150" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>160.2_TL_CUENERA_0_T_23</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>Cuenta Financiera en USD</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B152" s="5" t="inlineStr">
+        <is>
+          <t>160.2_AVOS_RERVA_0_T_15</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>Activos de Reserva en USD</t>
+        </is>
+      </c>
+      <c r="D152" s="5" t="inlineStr">
+        <is>
+          <t>BALANZA DE PAGOS T</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>161.1_TL_DEUDRNA_0_0_19</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>Deuda Externa Bruta Total en USD</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>DEUDA EXTERNA T</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>Sector Externo: Apendice5</t>
+        </is>
+      </c>
+      <c r="B154" s="5" t="inlineStr">
+        <is>
+          <t>313.1_TOTALTAL_0_T_5</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>Deuda Externa Bruta Privada en USD</t>
+        </is>
+      </c>
+      <c r="D154" s="5" t="inlineStr">
+        <is>
+          <t>DEUDA EXTERNA T</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>89.2_TS_INTELAR_0_D_20</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>Tasa BADLAR</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>8.1 Tasas de interes D</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B156" s="5" t="inlineStr">
+        <is>
+          <t>90.1_BMT_0_0_20</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>Base Monetaria (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D156" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>90.1_BMCMT_0_0_42</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>Circulación monetaria (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B158" s="5" t="inlineStr">
+        <is>
+          <t>90.1_BMCCB_0_0_36</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>Cuenta Corriente en el BCRA (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D158" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>90.1_AMTM2_0_0_31</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>M2 (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B160" s="5" t="inlineStr">
+        <is>
+          <t>90.1_AMTM3_0_0_31</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>M3 (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D160" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DTPPUB_0_0_31</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos en pesos (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B162" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DTPPRI_0_0_31</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos en pesos del sector privado (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D162" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DTPT_0_0_29</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos en pesos del sector público (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D163" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B164" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DTDPUB_0_0_33</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos en dólares (Millones de USD)</t>
+        </is>
+      </c>
+      <c r="D164" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DTDPRI_0_0_33</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos en dólares del sector privado (Millones de USD)</t>
+        </is>
+      </c>
+      <c r="D165" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B166" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DTDT_0_0_31</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos en dólares del sector público (Millones de USD)</t>
+        </is>
+      </c>
+      <c r="D166" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DET_DESAGRTAL_0_0_38</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos a plazo en pesos y dólares (Personales + Tarjetas) (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D167" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B168" s="5" t="inlineStr">
+        <is>
+          <t>90.1_DET_DESAGRTAL_0_0_44</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Depósitos a plazo en pesos (Personales + Tarjetas) (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D168" s="5" t="inlineStr">
+        <is>
+          <t>8.2 Agregados monetarios M</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>91.1_PEFPC_0_0_35</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>Préstamos al sector privado en pesos y dólares (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D169" s="5" t="inlineStr">
+        <is>
+          <t>8.3 Prest. de Entidades finac. M</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B170" s="5" t="inlineStr">
+        <is>
+          <t>91.1_DETALLE_PRPOT_0_0_25</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Préstamos al sector privado en pesos (Millones de $)</t>
+        </is>
+      </c>
+      <c r="D170" s="5" t="inlineStr">
+        <is>
+          <t>8.3 Prest. de Entidades finac. M</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>92.2_RESERVAS_IRES_0_0_32_40</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>Reservas Internacionales del BCRA (En mill. USD)</t>
+        </is>
+      </c>
+      <c r="D171" s="5" t="inlineStr">
+        <is>
+          <t>8.4 Res. Int. y Pasivos BCRA D</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B172" s="5" t="inlineStr">
+        <is>
+          <t>92.2_PASIVOS_MOIOS_0_0_18_34</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>Pasivos Monetarios</t>
+        </is>
+      </c>
+      <c r="D172" s="5" t="inlineStr">
+        <is>
+          <t>8.4 Res. Int. y Pasivos BCRA D</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>92.2_PASIVOS_MOSOS_0_0_31_15</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>Letras del BCRA. Saldo en Pesos</t>
+        </is>
+      </c>
+      <c r="D173" s="5" t="inlineStr">
+        <is>
+          <t>8.4 Res. Int. y Pasivos BCRA D</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B174" s="5" t="inlineStr">
+        <is>
+          <t>92.2_PASIVOS_MORES_0_0_33_100</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>Letras del BCRA. Saldo en Dólares</t>
+        </is>
+      </c>
+      <c r="D174" s="5" t="inlineStr">
+        <is>
+          <t>8.4 Res. Int. y Pasivos BCRA D</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>92.2_OTROS_DEPORNO_0_0_24_42</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>Otros Depósitos del Gobierno</t>
+        </is>
+      </c>
+      <c r="D175" s="5" t="inlineStr">
+        <is>
+          <t>8.4 Res. Int. y Pasivos BCRA D</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B176" s="5" t="inlineStr">
+        <is>
+          <t>92.2_TIPO_CAMBIION_0_0_21_24</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>Tipo de cambio ($/USD)</t>
+        </is>
+      </c>
+      <c r="D176" s="5" t="inlineStr">
+        <is>
+          <t>8.4 Res. Int. y Pasivos BCRA D</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>94.2_CD_D_0_0_10</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="D177" s="5" t="inlineStr">
+        <is>
+          <t>8.6 CER, UVA y UVI D</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="28.8" customHeight="1">
+      <c r="A178" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B178" s="5" t="inlineStr">
+        <is>
+          <t>94.2_UVAD_D_0_0_10</t>
+        </is>
+      </c>
+      <c r="C178" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UVA 
+</t>
+        </is>
+      </c>
+      <c r="D178" s="5" t="inlineStr">
+        <is>
+          <t>8.6 CER, UVA y UVI D</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B179" s="5" t="inlineStr">
+        <is>
+          <t>175.1_DR_ESTANSE_0_0_20</t>
+        </is>
+      </c>
+      <c r="C179" s="5" t="inlineStr">
+        <is>
+          <t>Dolar Estadounidense</t>
+        </is>
+      </c>
+      <c r="D179" s="5" t="inlineStr">
+        <is>
+          <t>8.8. Tipos de cambio historicos D</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="28.8" customHeight="1">
+      <c r="A180" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>175.1_DR_REFE500_0_0_25</t>
+        </is>
+      </c>
+      <c r="C180" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dolar Referencia Com 3500
+</t>
+        </is>
+      </c>
+      <c r="D180" s="5" t="inlineStr">
+        <is>
+          <t>8.8. Tipos de cambio historicos D</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B181" s="5" t="inlineStr">
+        <is>
+          <t>331.2_SALDO_BASERIA__15</t>
+        </is>
+      </c>
+      <c r="C181" s="5" t="inlineStr">
+        <is>
+          <t>Saldo Base Monetaria</t>
+        </is>
+      </c>
+      <c r="D181" s="5" t="inlineStr">
+        <is>
+          <t>8.11 Factores Base Monetaria D</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="43.2" customHeight="1">
+      <c r="A182" s="5" t="inlineStr">
+        <is>
+          <t>Dinero y Bancos: Apendice8</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>331.2_TOTAL_VARIION__27</t>
+        </is>
+      </c>
+      <c r="C182" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total variación de Saldo Base Monetaria
+</t>
+        </is>
+      </c>
+      <c r="D182" s="5" t="inlineStr">
+        <is>
+          <t>8.11 Factores Base Monetaria D</t>
         </is>
       </c>
     </row>

</xml_diff>